<commit_message>
Paraffin oil aquatox from three 2026 conclusion
Until we understand the differences between the different kinds of
paraffin oil we treat them as equivalent.
</commit_message>
<xml_diff>
--- a/data_generation/10_aquatic_toxicity/paraffin_oil_aquatic_toxicity.xlsx
+++ b/data_generation/10_aquatic_toxicity/paraffin_oil_aquatic_toxicity.xlsx
@@ -5,18 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Data-Work\41_AssessmentPPP-RE\412.34_Projekte\054_derappp\05_Daten\Input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Data-Work\41_AssessmentPPP-RE\412.34_Projekte\054_derappp\05_Daten\Input\10_aquatic_toxicity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0892D925-4949-4D13-8635-80AD8CBB737E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EF4F447-0C13-4F20-AFC7-86C43F92AC52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aquatic toxicity" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Aquatic toxicity'!$A$1:$V$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Aquatic toxicity'!$A$1:$V$31</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="86">
   <si>
     <t>substance</t>
   </si>
@@ -189,9 +189,6 @@
     <t>static</t>
   </si>
   <si>
-    <t>geomean</t>
-  </si>
-  <si>
     <t>35 d</t>
   </si>
   <si>
@@ -217,13 +214,85 @@
   </si>
   <si>
     <t>j.efsa.2024.8913_LoEP</t>
+  </si>
+  <si>
+    <t>OLIE-H</t>
+  </si>
+  <si>
+    <t>Culex sp.</t>
+  </si>
+  <si>
+    <t>17 d</t>
+  </si>
+  <si>
+    <t>mg/m2</t>
+  </si>
+  <si>
+    <t>FALSE</t>
+  </si>
+  <si>
+    <t>CAS 64742-46-7, chain lengths C16-C25</t>
+  </si>
+  <si>
+    <t>luel</t>
+  </si>
+  <si>
+    <t>Notonecta sp.</t>
+  </si>
+  <si>
+    <t>μg/L</t>
+  </si>
+  <si>
+    <t>TRUE</t>
+  </si>
+  <si>
+    <t>CITROLE</t>
+  </si>
+  <si>
+    <t>28 d</t>
+  </si>
+  <si>
+    <t>im</t>
+  </si>
+  <si>
+    <t>Polithiol</t>
+  </si>
+  <si>
+    <t>j.efsa.2026.9866</t>
+  </si>
+  <si>
+    <t>CAS 97862-82-3, chain lengths C16-C28</t>
+  </si>
+  <si>
+    <t>j.efsa.2026.9867</t>
+  </si>
+  <si>
+    <t>CAS 7262-86-0</t>
+  </si>
+  <si>
+    <t>gmm</t>
+  </si>
+  <si>
+    <t>Endpoint already recorded from j.efsa.2026.9867</t>
+  </si>
+  <si>
+    <t>j.efsa.2026.9868</t>
+  </si>
+  <si>
+    <t>Unit not convertible to concentration units</t>
+  </si>
+  <si>
+    <t>Unit not convertible to concentration units; Endpoint already recorded from j.efsa.2026.9867</t>
+  </si>
+  <si>
+    <t>EFSA LoEP. Product contains sulfur as second active ingredient. As endpoints are "greater than" endpoints, they are still valid as lower bounds.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -236,6 +305,14 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -258,11 +335,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -559,32 +640,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:V31"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.7265625" customWidth="1"/>
-    <col min="2" max="2" width="22.7265625" customWidth="1"/>
-    <col min="3" max="3" width="31.7265625" customWidth="1"/>
-    <col min="4" max="4" width="7.7265625" customWidth="1"/>
-    <col min="5" max="5" width="11.7265625" customWidth="1"/>
-    <col min="6" max="6" width="19.7265625" customWidth="1"/>
-    <col min="7" max="7" width="8.7265625" customWidth="1"/>
-    <col min="8" max="8" width="10.7265625" customWidth="1"/>
-    <col min="9" max="9" width="11.7265625" customWidth="1"/>
-    <col min="10" max="10" width="14.7265625" customWidth="1"/>
-    <col min="11" max="11" width="5.7265625" customWidth="1"/>
-    <col min="12" max="12" width="4.7265625" customWidth="1"/>
-    <col min="13" max="13" width="5.7265625" customWidth="1"/>
-    <col min="14" max="14" width="4.7265625" customWidth="1"/>
-    <col min="15" max="15" width="8.7265625" customWidth="1"/>
-    <col min="16" max="16" width="16.7265625" customWidth="1"/>
-    <col min="17" max="17" width="4.7265625" customWidth="1"/>
-    <col min="18" max="18" width="8.7265625" customWidth="1"/>
-    <col min="19" max="19" width="9.7265625" customWidth="1"/>
-    <col min="20" max="20" width="4.7265625" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="3" width="31.7109375" customWidth="1"/>
+    <col min="4" max="4" width="7.7109375" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" customWidth="1"/>
+    <col min="6" max="6" width="19.7109375" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" customWidth="1"/>
+    <col min="9" max="9" width="11.7109375" customWidth="1"/>
+    <col min="10" max="10" width="14.7109375" customWidth="1"/>
+    <col min="11" max="11" width="5.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="5.7109375" customWidth="1"/>
+    <col min="14" max="14" width="4.7109375" customWidth="1"/>
+    <col min="15" max="15" width="8.7109375" customWidth="1"/>
+    <col min="16" max="16" width="16.7109375" customWidth="1"/>
+    <col min="17" max="17" width="4.7109375" customWidth="1"/>
+    <col min="18" max="18" width="8.7109375" customWidth="1"/>
+    <col min="19" max="19" width="9.7109375" customWidth="1"/>
+    <col min="20" max="20" width="10.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -652,7 +733,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>22</v>
       </c>
@@ -690,13 +771,13 @@
         <v>50</v>
       </c>
       <c r="P2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Q2">
         <v>70</v>
       </c>
-      <c r="R2" t="b">
-        <v>1</v>
+      <c r="R2" t="s">
+        <v>71</v>
       </c>
       <c r="S2" t="s">
         <v>29</v>
@@ -708,7 +789,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>22</v>
       </c>
@@ -743,16 +824,16 @@
         <v>28</v>
       </c>
       <c r="O3" t="s">
-        <v>53</v>
+        <v>80</v>
       </c>
       <c r="P3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Q3">
         <v>70</v>
       </c>
-      <c r="R3" t="b">
-        <v>1</v>
+      <c r="R3" t="s">
+        <v>71</v>
       </c>
       <c r="S3" t="s">
         <v>29</v>
@@ -764,7 +845,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -802,13 +883,13 @@
         <v>50</v>
       </c>
       <c r="P4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Q4">
         <v>70</v>
       </c>
-      <c r="R4" t="b">
-        <v>1</v>
+      <c r="R4" t="s">
+        <v>71</v>
       </c>
       <c r="S4" t="s">
         <v>29</v>
@@ -820,7 +901,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>22</v>
       </c>
@@ -837,10 +918,10 @@
         <v>48</v>
       </c>
       <c r="G5" t="s">
+        <v>53</v>
+      </c>
+      <c r="H5" t="s">
         <v>54</v>
-      </c>
-      <c r="H5" t="s">
-        <v>55</v>
       </c>
       <c r="K5" t="s">
         <v>35</v>
@@ -858,13 +939,13 @@
         <v>50</v>
       </c>
       <c r="P5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Q5">
         <v>70</v>
       </c>
-      <c r="R5" t="b">
-        <v>1</v>
+      <c r="R5" t="s">
+        <v>71</v>
       </c>
       <c r="S5" t="s">
         <v>29</v>
@@ -876,7 +957,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>22</v>
       </c>
@@ -893,10 +974,10 @@
         <v>52</v>
       </c>
       <c r="G6" t="s">
+        <v>55</v>
+      </c>
+      <c r="I6" t="s">
         <v>56</v>
-      </c>
-      <c r="I6" t="s">
-        <v>57</v>
       </c>
       <c r="K6" t="s">
         <v>38</v>
@@ -911,16 +992,16 @@
         <v>28</v>
       </c>
       <c r="O6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="P6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Q6">
         <v>70</v>
       </c>
-      <c r="R6" t="b">
-        <v>1</v>
+      <c r="R6" t="s">
+        <v>71</v>
       </c>
       <c r="S6" t="s">
         <v>29</v>
@@ -932,7 +1013,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -949,10 +1030,10 @@
         <v>48</v>
       </c>
       <c r="G7" t="s">
+        <v>55</v>
+      </c>
+      <c r="I7" t="s">
         <v>56</v>
-      </c>
-      <c r="I7" t="s">
-        <v>57</v>
       </c>
       <c r="K7" t="s">
         <v>38</v>
@@ -970,13 +1051,13 @@
         <v>50</v>
       </c>
       <c r="P7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Q7">
         <v>70</v>
       </c>
-      <c r="R7" t="b">
-        <v>1</v>
+      <c r="R7" t="s">
+        <v>71</v>
       </c>
       <c r="S7" t="s">
         <v>29</v>
@@ -988,7 +1069,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -1002,10 +1083,10 @@
         <v>7</v>
       </c>
       <c r="G8" t="s">
+        <v>55</v>
+      </c>
+      <c r="I8" t="s">
         <v>56</v>
-      </c>
-      <c r="I8" t="s">
-        <v>57</v>
       </c>
       <c r="K8" t="s">
         <v>38</v>
@@ -1023,13 +1104,13 @@
         <v>50</v>
       </c>
       <c r="P8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Q8">
         <v>70</v>
       </c>
-      <c r="R8" t="b">
-        <v>1</v>
+      <c r="R8" t="s">
+        <v>71</v>
       </c>
       <c r="S8" t="s">
         <v>29</v>
@@ -1041,7 +1122,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -1055,10 +1136,10 @@
         <v>48</v>
       </c>
       <c r="G9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J9" t="s">
         <v>40</v>
@@ -1079,13 +1160,13 @@
         <v>50</v>
       </c>
       <c r="P9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Q9">
         <v>70</v>
       </c>
-      <c r="R9" t="b">
-        <v>1</v>
+      <c r="R9" t="s">
+        <v>71</v>
       </c>
       <c r="S9" t="s">
         <v>29</v>
@@ -1097,7 +1178,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1111,10 +1192,10 @@
         <v>48</v>
       </c>
       <c r="G10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J10" t="s">
         <v>40</v>
@@ -1135,13 +1216,13 @@
         <v>50</v>
       </c>
       <c r="P10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Q10">
         <v>70</v>
       </c>
-      <c r="R10" t="b">
-        <v>1</v>
+      <c r="R10" t="s">
+        <v>71</v>
       </c>
       <c r="S10" t="s">
         <v>29</v>
@@ -1153,7 +1234,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -1167,7 +1248,7 @@
         <v>9</v>
       </c>
       <c r="G11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K11" t="s">
         <v>35</v>
@@ -1185,13 +1266,13 @@
         <v>50</v>
       </c>
       <c r="P11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Q11">
         <v>70</v>
       </c>
-      <c r="R11" t="b">
-        <v>1</v>
+      <c r="R11" t="s">
+        <v>71</v>
       </c>
       <c r="S11" t="s">
         <v>29</v>
@@ -1203,7 +1284,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -1220,7 +1301,7 @@
         <v>52</v>
       </c>
       <c r="G12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K12" t="s">
         <v>38</v>
@@ -1235,13 +1316,13 @@
         <v>28</v>
       </c>
       <c r="P12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Q12">
         <v>70</v>
       </c>
-      <c r="R12" t="b">
-        <v>1</v>
+      <c r="R12" t="s">
+        <v>71</v>
       </c>
       <c r="S12" t="s">
         <v>29</v>
@@ -1253,7 +1334,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1267,7 +1348,7 @@
         <v>11</v>
       </c>
       <c r="G13" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K13" t="s">
         <v>38</v>
@@ -1285,13 +1366,13 @@
         <v>50</v>
       </c>
       <c r="P13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Q13">
         <v>70</v>
       </c>
-      <c r="R13" t="b">
-        <v>1</v>
+      <c r="R13" t="s">
+        <v>71</v>
       </c>
       <c r="S13" t="s">
         <v>29</v>
@@ -1303,7 +1384,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>22</v>
       </c>
@@ -1320,7 +1401,7 @@
         <v>52</v>
       </c>
       <c r="G14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I14" t="s">
         <v>45</v>
@@ -1341,13 +1422,13 @@
         <v>50</v>
       </c>
       <c r="P14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Q14">
         <v>70</v>
       </c>
-      <c r="R14" t="b">
-        <v>1</v>
+      <c r="R14" t="s">
+        <v>71</v>
       </c>
       <c r="S14" t="s">
         <v>29</v>
@@ -1359,7 +1440,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -1376,7 +1457,7 @@
         <v>52</v>
       </c>
       <c r="G15" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I15" t="s">
         <v>46</v>
@@ -1397,13 +1478,13 @@
         <v>50</v>
       </c>
       <c r="P15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Q15">
         <v>70</v>
       </c>
-      <c r="R15" t="b">
-        <v>1</v>
+      <c r="R15" t="s">
+        <v>71</v>
       </c>
       <c r="S15" t="s">
         <v>29</v>
@@ -1415,7 +1496,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -1429,7 +1510,7 @@
         <v>13</v>
       </c>
       <c r="G16" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I16" t="s">
         <v>45</v>
@@ -1450,13 +1531,13 @@
         <v>50</v>
       </c>
       <c r="P16" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Q16">
         <v>70</v>
       </c>
-      <c r="R16" t="b">
-        <v>1</v>
+      <c r="R16" t="s">
+        <v>71</v>
       </c>
       <c r="S16" t="s">
         <v>29</v>
@@ -1468,8 +1549,859 @@
         <v>51</v>
       </c>
     </row>
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D17" s="2">
+        <v>1</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M17" s="2">
+        <v>135.69999999999999</v>
+      </c>
+      <c r="N17" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="O17" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="P17" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q17" s="2">
+        <v>40</v>
+      </c>
+      <c r="R17" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="S17" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="T17" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="U17" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="V17" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D18" s="2">
+        <v>2</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M18" s="2">
+        <v>32</v>
+      </c>
+      <c r="N18" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="O18" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="P18" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q18" s="2">
+        <v>40</v>
+      </c>
+      <c r="R18" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="S18" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="T18" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="U18" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="V18" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C19" t="s">
+        <v>47</v>
+      </c>
+      <c r="D19" s="2">
+        <v>3</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I19" t="s">
+        <v>60</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L19" t="s">
+        <v>32</v>
+      </c>
+      <c r="M19">
+        <v>35500</v>
+      </c>
+      <c r="N19" t="s">
+        <v>70</v>
+      </c>
+      <c r="O19" t="s">
+        <v>80</v>
+      </c>
+      <c r="P19" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q19" s="2">
+        <v>40</v>
+      </c>
+      <c r="R19" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="S19" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="T19" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="U19" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="V19" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C20" t="s">
+        <v>47</v>
+      </c>
+      <c r="D20" s="2">
+        <v>3</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="L20" t="s">
+        <v>27</v>
+      </c>
+      <c r="M20">
+        <v>7680</v>
+      </c>
+      <c r="N20" t="s">
+        <v>70</v>
+      </c>
+      <c r="O20" t="s">
+        <v>80</v>
+      </c>
+      <c r="P20" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q20" s="2">
+        <v>40</v>
+      </c>
+      <c r="R20" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="S20" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="T20" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="U20" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="V20" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" t="s">
+        <v>72</v>
+      </c>
+      <c r="C21" t="s">
+        <v>43</v>
+      </c>
+      <c r="D21" s="2">
+        <v>4</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="L21" t="s">
+        <v>27</v>
+      </c>
+      <c r="M21">
+        <v>752</v>
+      </c>
+      <c r="N21" t="s">
+        <v>70</v>
+      </c>
+      <c r="O21" t="s">
+        <v>74</v>
+      </c>
+      <c r="P21" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q21" s="2">
+        <v>40</v>
+      </c>
+      <c r="R21" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="S21" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="T21" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="U21" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="V21" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D22" s="2">
+        <v>5</v>
+      </c>
+      <c r="G22" t="s">
+        <v>49</v>
+      </c>
+      <c r="K22" t="s">
+        <v>26</v>
+      </c>
+      <c r="L22" t="s">
+        <v>32</v>
+      </c>
+      <c r="M22" s="3">
+        <v>153</v>
+      </c>
+      <c r="N22" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="O22" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="P22" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q22" s="2">
+        <v>39</v>
+      </c>
+      <c r="R22" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="S22" t="s">
+        <v>85</v>
+      </c>
+      <c r="T22" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="U22" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="V22" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C23" t="s">
+        <v>47</v>
+      </c>
+      <c r="D23" s="2">
+        <v>6</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I23" t="s">
+        <v>46</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L23" t="s">
+        <v>32</v>
+      </c>
+      <c r="M23">
+        <v>167</v>
+      </c>
+      <c r="N23" t="s">
+        <v>28</v>
+      </c>
+      <c r="O23" t="s">
+        <v>80</v>
+      </c>
+      <c r="P23" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q23" s="2">
+        <v>39</v>
+      </c>
+      <c r="R23" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="S23" t="s">
+        <v>85</v>
+      </c>
+      <c r="T23" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="U23" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="V23" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C24" t="s">
+        <v>47</v>
+      </c>
+      <c r="D24" s="2">
+        <v>6</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I24" t="s">
+        <v>60</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L24" t="s">
+        <v>32</v>
+      </c>
+      <c r="M24">
+        <v>167</v>
+      </c>
+      <c r="N24" t="s">
+        <v>28</v>
+      </c>
+      <c r="O24" t="s">
+        <v>80</v>
+      </c>
+      <c r="P24" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q24" s="2">
+        <v>39</v>
+      </c>
+      <c r="R24" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="S24" t="s">
+        <v>85</v>
+      </c>
+      <c r="T24" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="U24" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="V24" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>22</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C25" t="s">
+        <v>47</v>
+      </c>
+      <c r="D25" s="2">
+        <v>7</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I25" t="s">
+        <v>46</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L25" t="s">
+        <v>32</v>
+      </c>
+      <c r="M25">
+        <v>100</v>
+      </c>
+      <c r="N25" t="s">
+        <v>28</v>
+      </c>
+      <c r="O25" t="s">
+        <v>57</v>
+      </c>
+      <c r="P25" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q25" s="2">
+        <v>39</v>
+      </c>
+      <c r="R25" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="S25" t="s">
+        <v>85</v>
+      </c>
+      <c r="T25" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="U25" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="V25" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>22</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C26" t="s">
+        <v>47</v>
+      </c>
+      <c r="D26" s="2">
+        <v>7</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I26" t="s">
+        <v>60</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L26" t="s">
+        <v>32</v>
+      </c>
+      <c r="M26">
+        <v>100</v>
+      </c>
+      <c r="N26" t="s">
+        <v>28</v>
+      </c>
+      <c r="O26" t="s">
+        <v>57</v>
+      </c>
+      <c r="P26" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q26" s="2">
+        <v>39</v>
+      </c>
+      <c r="R26" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="S26" t="s">
+        <v>85</v>
+      </c>
+      <c r="T26" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="U26" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="V26" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>22</v>
+      </c>
+      <c r="B27" t="s">
+        <v>62</v>
+      </c>
+      <c r="C27" t="s">
+        <v>63</v>
+      </c>
+      <c r="D27" s="2">
+        <v>8</v>
+      </c>
+      <c r="E27" t="s">
+        <v>52</v>
+      </c>
+      <c r="G27" t="s">
+        <v>64</v>
+      </c>
+      <c r="K27" t="s">
+        <v>38</v>
+      </c>
+      <c r="L27" t="s">
+        <v>27</v>
+      </c>
+      <c r="M27">
+        <v>135.69999999999999</v>
+      </c>
+      <c r="N27" t="s">
+        <v>65</v>
+      </c>
+      <c r="O27" t="s">
+        <v>50</v>
+      </c>
+      <c r="P27" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q27" s="2">
+        <v>45</v>
+      </c>
+      <c r="R27" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="S27" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="T27" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="U27" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="V27" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>22</v>
+      </c>
+      <c r="B28" t="s">
+        <v>62</v>
+      </c>
+      <c r="C28" t="s">
+        <v>69</v>
+      </c>
+      <c r="D28" s="2">
+        <v>9</v>
+      </c>
+      <c r="E28" t="s">
+        <v>52</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L28" t="s">
+        <v>27</v>
+      </c>
+      <c r="M28">
+        <v>32.5</v>
+      </c>
+      <c r="N28" t="s">
+        <v>65</v>
+      </c>
+      <c r="O28" t="s">
+        <v>50</v>
+      </c>
+      <c r="P28" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q28" s="2">
+        <v>45</v>
+      </c>
+      <c r="R28" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="S28" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="T28" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="U28" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="V28" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>22</v>
+      </c>
+      <c r="B29" t="s">
+        <v>62</v>
+      </c>
+      <c r="C29" t="s">
+        <v>47</v>
+      </c>
+      <c r="D29" s="2">
+        <v>10</v>
+      </c>
+      <c r="E29" t="s">
+        <v>52</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I29" t="s">
+        <v>60</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L29" t="s">
+        <v>32</v>
+      </c>
+      <c r="M29">
+        <v>35500</v>
+      </c>
+      <c r="N29" t="s">
+        <v>70</v>
+      </c>
+      <c r="O29" t="s">
+        <v>80</v>
+      </c>
+      <c r="P29" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q29" s="2">
+        <v>45</v>
+      </c>
+      <c r="R29" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="S29" s="2"/>
+      <c r="T29" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="U29" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="V29" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>22</v>
+      </c>
+      <c r="B30" t="s">
+        <v>62</v>
+      </c>
+      <c r="C30" t="s">
+        <v>47</v>
+      </c>
+      <c r="D30" s="2">
+        <v>10</v>
+      </c>
+      <c r="E30" t="s">
+        <v>52</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="L30" t="s">
+        <v>27</v>
+      </c>
+      <c r="M30">
+        <v>7680</v>
+      </c>
+      <c r="N30" t="s">
+        <v>70</v>
+      </c>
+      <c r="O30" t="s">
+        <v>80</v>
+      </c>
+      <c r="P30" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q30" s="2">
+        <v>45</v>
+      </c>
+      <c r="R30" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="S30" s="2"/>
+      <c r="T30" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="U30" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="V30" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>22</v>
+      </c>
+      <c r="B31" t="s">
+        <v>72</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31" s="2">
+        <v>11</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="L31" t="s">
+        <v>27</v>
+      </c>
+      <c r="M31">
+        <v>752</v>
+      </c>
+      <c r="N31" t="s">
+        <v>70</v>
+      </c>
+      <c r="O31" t="s">
+        <v>74</v>
+      </c>
+      <c r="P31" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q31" s="2">
+        <v>45</v>
+      </c>
+      <c r="R31" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="S31" s="2"/>
+      <c r="T31" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="U31" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="V31" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:V16" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:V31" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix numbering of paraffin oil tests
</commit_message>
<xml_diff>
--- a/data_generation/10_aquatic_toxicity/paraffin_oil_aquatic_toxicity.xlsx
+++ b/data_generation/10_aquatic_toxicity/paraffin_oil_aquatic_toxicity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Data-Work\41_AssessmentPPP-RE\412.34_Projekte\054_derappp\05_Daten\Input\10_aquatic_toxicity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EF4F447-0C13-4F20-AFC7-86C43F92AC52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D6C9F10-EE5F-49F2-9A17-CC0A69C188D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1560,7 +1560,7 @@
         <v>63</v>
       </c>
       <c r="D17" s="2">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>52</v>
@@ -1620,7 +1620,7 @@
         <v>69</v>
       </c>
       <c r="D18" s="2">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>52</v>
@@ -1680,7 +1680,7 @@
         <v>47</v>
       </c>
       <c r="D19" s="2">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>52</v>
@@ -1739,7 +1739,7 @@
         <v>47</v>
       </c>
       <c r="D20" s="2">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>52</v>
@@ -1795,7 +1795,7 @@
         <v>43</v>
       </c>
       <c r="D21" s="2">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>73</v>
@@ -1848,7 +1848,7 @@
         <v>24</v>
       </c>
       <c r="D22" s="2">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="G22" t="s">
         <v>49</v>
@@ -1901,7 +1901,7 @@
         <v>47</v>
       </c>
       <c r="D23" s="2">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>52</v>
@@ -1960,7 +1960,7 @@
         <v>47</v>
       </c>
       <c r="D24" s="2">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>52</v>
@@ -2019,7 +2019,7 @@
         <v>47</v>
       </c>
       <c r="D25" s="2">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>48</v>
@@ -2078,7 +2078,7 @@
         <v>47</v>
       </c>
       <c r="D26" s="2">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>48</v>
@@ -2137,7 +2137,7 @@
         <v>63</v>
       </c>
       <c r="D27" s="2">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="E27" t="s">
         <v>52</v>
@@ -2193,7 +2193,7 @@
         <v>69</v>
       </c>
       <c r="D28" s="2">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="E28" t="s">
         <v>52</v>
@@ -2249,7 +2249,7 @@
         <v>47</v>
       </c>
       <c r="D29" s="2">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="E29" t="s">
         <v>52</v>
@@ -2306,7 +2306,7 @@
         <v>47</v>
       </c>
       <c r="D30" s="2">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="E30" t="s">
         <v>52</v>
@@ -2360,7 +2360,7 @@
         <v>43</v>
       </c>
       <c r="D31" s="2">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>73</v>

</xml_diff>